<commit_message>
Use jirai embbeding model as main result folder
</commit_message>
<xml_diff>
--- a/data/censo_escolar_dataset/augmentation_method_results/censo_escolar_algorithm_only_augmented_semantic_variation.xlsx
+++ b/data/censo_escolar_dataset/augmentation_method_results/censo_escolar_algorithm_only_augmented_semantic_variation.xlsx
@@ -770,10 +770,10 @@
         <v>107</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.2081575932284499</v>
+        <v>0.1631942729772794</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.2074868765679451</v>
+        <v>0.1581419594434759</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -853,31 +853,31 @@
         <v>107</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0.00545572229427993</v>
+        <v>0.001542117467544957</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.3910181333423479</v>
+        <v>0.1603287581480964</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.1234734910515997</v>
+        <v>0.05656259379032474</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.1243673807309887</v>
+        <v>0.04908215245058689</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.08220190689467777</v>
+        <v>0.03846191027440449</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.05772578043056709</v>
+        <v>0.02183253542619557</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0.1745244683799224</v>
+        <v>0.07631411628191997</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.2239010850483072</v>
+        <v>0.1110788129464591</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.2685969939528372</v>
+        <v>0.1288999210502582</v>
       </c>
     </row>
     <row r="12">
@@ -893,28 +893,28 @@
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.5980001585399306</v>
+        <v>0.5897443458289537</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.2928416954053001</v>
+        <v>0.269825952164234</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.2893310685673767</v>
+        <v>0.253719552315225</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.1380787811628306</v>
+        <v>0.1362561754252902</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.1934311829674767</v>
+        <v>0.1689655062940617</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.4169755438730119</v>
+        <v>0.3394929829036214</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.4798551468116325</v>
+        <v>0.4583073191389085</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0.5179365739053469</v>
+        <v>0.5238216532112895</v>
       </c>
     </row>
     <row r="13">
@@ -927,31 +927,31 @@
         <v>107</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.002727861147139965</v>
+        <v>0.0007710587337724784</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.4288962694812777</v>
+        <v>0.3542423960307823</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.2081575932284499</v>
+        <v>0.1631942729772794</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.2074868765679451</v>
+        <v>0.1581419594434759</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.1026092892442432</v>
+        <v>0.08068154794158187</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.1333465229488505</v>
+        <v>0.1070369975673368</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0.282991928406626</v>
+        <v>0.2051346624288827</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.3473885284365502</v>
+        <v>0.2831184907778132</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.3666953184780288</v>
+        <v>0.2952907867489171</v>
       </c>
     </row>
     <row r="15">
@@ -1003,16 +1003,16 @@
         <v>29</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0.2042491006714809</v>
+        <v>0.1492057110643492</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.2074868765679451</v>
+        <v>0.1342486012739472</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.305457745711989</v>
+        <v>0.235060871513743</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.3278790416438995</v>
+        <v>0.2543464342920197</v>
       </c>
     </row>
     <row r="18">
@@ -1025,16 +1025,16 @@
         <v>46</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>0.2709665944958294</v>
+        <v>0.2142353911724133</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.2785366868192118</v>
+        <v>0.2031549971515484</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.3661890581184134</v>
+        <v>0.3014089144549226</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.3863337994960723</v>
+        <v>0.3297016080637158</v>
       </c>
     </row>
     <row r="19">
@@ -1047,16 +1047,16 @@
         <v>8</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0.1093009836649237</v>
+        <v>0.08948904752893939</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.1242955210963803</v>
+        <v>0.1139643095327257</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.2034114750721504</v>
+        <v>0.1731453436174966</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.2356230633501135</v>
+        <v>0.1770600870636711</v>
       </c>
     </row>
     <row r="20">
@@ -1069,16 +1069,16 @@
         <v>24</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>0.1254486391601524</v>
+        <v>0.1068367172308434</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0.1154110347512379</v>
+        <v>0.09751510346577935</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.2038654423705859</v>
+        <v>0.157933576800706</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.2092828187591739</v>
+        <v>0.1670905129788623</v>
       </c>
     </row>
   </sheetData>
@@ -1211,31 +1211,31 @@
         <v>29</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.009177108301621995</v>
+        <v>0.01277945069268038</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.2781696602568258</v>
+        <v>0.1081172332545961</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.1186384310366887</v>
+        <v>0.04772795854439046</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1158273980785529</v>
+        <v>0.04582844888842386</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.06549497441926826</v>
+        <v>0.02303929925565545</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.07145806413193934</v>
+        <v>0.03365748656734324</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.144890272109781</v>
+        <v>0.06038194909204031</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>0.2139404786951167</v>
+        <v>0.07536087351104515</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>0.2314476896911405</v>
+        <v>0.08385852511933012</v>
       </c>
     </row>
     <row r="7">
@@ -1253,31 +1253,31 @@
         <v>29</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>1.028954699222595e-12</v>
+        <v>0</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.5058616126320689</v>
+        <v>0.4645084089213284</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.289859770306273</v>
+        <v>0.250683463584308</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.2939458194661031</v>
+        <v>0.2509656601952331</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.1159306337201217</v>
+        <v>0.1016900515332326</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.211841797297068</v>
+        <v>0.1838268447025366</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.3803718130735559</v>
+        <v>0.3105036685082296</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.4428200230351598</v>
+        <v>0.3989272617104594</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.4579272651340464</v>
+        <v>0.4206289863031082</v>
       </c>
     </row>
     <row r="8">
@@ -1295,31 +1295,31 @@
         <v>29</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.004588554151325475</v>
+        <v>0.02838366935883985</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.3920156364444473</v>
+        <v>0.2746769123757418</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.2042491006714809</v>
+        <v>0.1492057110643492</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.2074868765679451</v>
+        <v>0.1342486012739472</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.08399911173799099</v>
+        <v>0.05698392301866292</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.1416499307145037</v>
+        <v>0.1078844524143674</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.2801096918797846</v>
+        <v>0.1811762827892182</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0.305457745711989</v>
+        <v>0.235060871513743</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>0.3278790416438995</v>
+        <v>0.2543464342920197</v>
       </c>
     </row>
     <row r="9">
@@ -1337,31 +1337,31 @@
         <v>46</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.009565537910372179</v>
+        <v>0.003713459675007136</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.3910181333423479</v>
+        <v>0.1603287581480964</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.1706082649874723</v>
+        <v>0.07894051666884025</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.1652424473561811</v>
+        <v>0.07441569249673147</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0778031129380394</v>
+        <v>0.04054871877443127</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1307502416922228</v>
+        <v>0.04851857568305598</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.1917215648822679</v>
+        <v>0.1082302189397843</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>0.2636088449646325</v>
+        <v>0.1376874841630291</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>0.334014032184446</v>
+        <v>0.1546842335479116</v>
       </c>
     </row>
     <row r="10">
@@ -1379,31 +1379,31 @@
         <v>46</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1.145306072203311e-12</v>
+        <v>8.859579736508749e-14</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.5980001585399306</v>
+        <v>0.5897443458289537</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.3713249240041864</v>
+        <v>0.3495302656759863</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.3633637683532037</v>
+        <v>0.3338296894026354</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.126168459460737</v>
+        <v>0.1337327400056095</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0.3010758173933415</v>
+        <v>0.2656886054229249</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.4641932052113236</v>
+        <v>0.4478387701483538</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>0.5232805119902046</v>
+        <v>0.5319613733404924</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>0.5379770415961475</v>
+        <v>0.5625401551882124</v>
       </c>
     </row>
     <row r="11">
@@ -1421,31 +1421,31 @@
         <v>46</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.004782768955758743</v>
+        <v>0.001856729837547866</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.4288962694812777</v>
+        <v>0.3542423960307823</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.2709665944958294</v>
+        <v>0.2142353911724133</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.2785366868192118</v>
+        <v>0.2031549971515484</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.08964742757808788</v>
+        <v>0.07703876099732726</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0.2182240294417712</v>
+        <v>0.165917301965381</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.3421511605007387</v>
+        <v>0.2822834205204936</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0.3661890581184134</v>
+        <v>0.3014089144549226</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>0.3863337994960723</v>
+        <v>0.3297016080637158</v>
       </c>
     </row>
     <row r="12">
@@ -1463,31 +1463,31 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.00545572229427993</v>
+        <v>0.001542117467544957</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.1791718709407</v>
+        <v>0.06040171185460796</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.06633101558373386</v>
+        <v>0.02262775992148476</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.02940159876851112</v>
+        <v>0.01751056186704913</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.06697152526478276</v>
+        <v>0.01917898396804431</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.01263228083169204</v>
+        <v>0.009800898117648615</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.1201310174058536</v>
+        <v>0.02906051760851652</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0.1653313190251692</v>
+        <v>0.04980243269742485</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>0.1722515949829346</v>
+        <v>0.05510207227601641</v>
       </c>
     </row>
     <row r="13">
@@ -1508,28 +1508,28 @@
         <v>0</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.3564974323154532</v>
+        <v>0.3382889323707369</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.1522709517461135</v>
+        <v>0.156350335136394</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.189978122049498</v>
+        <v>0.1862276830167533</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.1274790103398517</v>
+        <v>0.1323192774257714</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>2.034261648020674e-12</v>
+        <v>0</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.2359724164858474</v>
+        <v>0.2452383108932948</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.2823874810437836</v>
+        <v>0.3252143462818626</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>0.3194424566796183</v>
+        <v>0.3317516393262997</v>
       </c>
     </row>
     <row r="14">
@@ -1547,31 +1547,31 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.002727861147139965</v>
+        <v>0.0007710587337724784</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.2678346516280766</v>
+        <v>0.1809748305098455</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.1093009836649237</v>
+        <v>0.08948904752893939</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.1242955210963803</v>
+        <v>0.1139643095327257</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.09175889677512811</v>
+        <v>0.07051870789190121</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>0.006316140416863153</v>
+        <v>0.006032513257144198</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.1707488866021626</v>
+        <v>0.1379752226836828</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>0.2034114750721504</v>
+        <v>0.1731453436174966</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>0.2356230633501135</v>
+        <v>0.1770600870636711</v>
       </c>
     </row>
     <row r="15">
@@ -1589,31 +1589,31 @@
         <v>24</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.007040395161529212</v>
+        <v>0.008911851635814538</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.1516533777556459</v>
+        <v>0.09387271445166978</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.05802169701514987</v>
+        <v>0.03565837048495391</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.04510738568599121</v>
+        <v>0.02003647955403265</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.04675766952150907</v>
+        <v>0.02837148796032184</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.01324953438740042</v>
+        <v>0.01484890304726086</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.09045782292299423</v>
+        <v>0.06010879710418413</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.1302781864953874</v>
+        <v>0.08576026129968224</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.1498117493697829</v>
+        <v>0.09194909249562835</v>
       </c>
     </row>
     <row r="16">
@@ -1631,31 +1631,31 @@
         <v>24</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.02220783922031455</v>
+        <v>0.03903781187129274</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.3431115613758197</v>
+        <v>0.3040846085479662</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.1928755813051549</v>
+        <v>0.1780150639767329</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1910413442066927</v>
+        <v>0.1689655062940617</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.06661512989430329</v>
+        <v>0.06944066427349463</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>0.158184461362114</v>
+        <v>0.1239730857237735</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.2383841610174764</v>
+        <v>0.2240161862487364</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0.2745928422505342</v>
+        <v>0.2707630229734116</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>0.29291778459743</v>
+        <v>0.2955086360078124</v>
       </c>
     </row>
     <row r="17">
@@ -1673,31 +1673,31 @@
         <v>24</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.01773629798773724</v>
+        <v>0.02589429983075525</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.2147448949250439</v>
+        <v>0.1980739750793566</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.1254486391601524</v>
+        <v>0.1068367172308434</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.1154110347512379</v>
+        <v>0.09751510346577935</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.05026282299763141</v>
+        <v>0.0429906036863878</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>0.08693934519052969</v>
+        <v>0.07353818825848264</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.1567008235021317</v>
+        <v>0.1371248050503327</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.2038654423705859</v>
+        <v>0.157933576800706</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.2092828187591739</v>
+        <v>0.1670905129788623</v>
       </c>
     </row>
   </sheetData>
@@ -1770,13 +1770,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -1786,13 +1786,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -1802,13 +1802,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D8" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1818,13 +1818,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1837,10 +1837,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1853,7 +1853,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -2023,13 +2023,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.00545572229427993</v>
+        <v>0.001542117467544957</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.002727861147139965</v>
+        <v>0.0007710587337724784</v>
       </c>
     </row>
     <row r="7">
@@ -2042,7 +2042,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2050,13 +2050,13 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.005899750453198682</v>
+        <v>0.003102973533906539</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>2.220446049250313e-16</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.002949875226599452</v>
+        <v>0.001551486766953269</v>
       </c>
     </row>
     <row r="8">
@@ -2069,21 +2069,21 @@
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Fácil</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.009177108301621995</v>
+        <v>0.003713459675007136</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.028954699222595e-12</v>
+        <v>8.859579736508749e-14</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.004588554151325475</v>
+        <v>0.001856729837547866</v>
       </c>
     </row>
     <row r="9">
@@ -2096,21 +2096,21 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Difícil</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.009565537910372179</v>
+        <v>0.01505237750774902</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>1.145306072203311e-12</v>
+        <v>0</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.004782768955758743</v>
+        <v>0.007526188753874508</v>
       </c>
     </row>
     <row r="10">
@@ -2123,21 +2123,21 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>12</v>
+        <v>106</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Difícil</t>
+          <t>Muito Difícil</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.01487645762452317</v>
+        <v>0.01275078779021777</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>2.712274849159257e-12</v>
+        <v>0.03903781187129274</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.00743822881361772</v>
+        <v>0.02589429983075525</v>
       </c>
     </row>
     <row r="11">
@@ -2150,21 +2150,21 @@
         <v>6</v>
       </c>
       <c r="C11" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Muito Difícil</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.01326475675515992</v>
+        <v>0.05676733871767969</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.02220783922031455</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.01773629798773724</v>
+        <v>0.02838366935883985</v>
       </c>
     </row>
     <row r="12">
@@ -2185,13 +2185,13 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.007817775614430089</v>
+        <v>0.01955819095508748</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.1089481461712205</v>
+        <v>0.07621519005436195</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.0583829608928253</v>
+        <v>0.04788669050472472</v>
       </c>
     </row>
     <row r="13">
@@ -2204,7 +2204,7 @@
         <v>8</v>
       </c>
       <c r="C13" t="n">
-        <v>86</v>
+        <v>15</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2212,13 +2212,13 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.04539817953123382</v>
+        <v>0.01888822568079318</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.1052228352000325</v>
+        <v>0.0848878560806775</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07531050736563316</v>
+        <v>0.05188804088073534</v>
       </c>
     </row>
     <row r="14">
@@ -2231,7 +2231,7 @@
         <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2239,13 +2239,13 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.008264539725053144</v>
+        <v>0.009567678282985548</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.1491662181009212</v>
+        <v>0.106159571735605</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.07871537891298719</v>
+        <v>0.05786362500929526</v>
       </c>
     </row>
     <row r="15">
@@ -2258,21 +2258,21 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Muito Difícil</t>
+          <t>Fácil</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.02008154682380892</v>
+        <v>0.01667131874915107</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.138105113781784</v>
+        <v>0.09979209920010135</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.07909333030279647</v>
+        <v>0.05823170897462621</v>
       </c>
     </row>
     <row r="16">
@@ -2285,7 +2285,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2293,13 +2293,13 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.3910181333423479</v>
+        <v>0.1187404462326108</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.4667744056202074</v>
+        <v>0.5897443458289537</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.4288962694812777</v>
+        <v>0.3542423960307823</v>
       </c>
     </row>
     <row r="17">
@@ -2312,7 +2312,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2320,13 +2320,13 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.3405401816638224</v>
+        <v>0.1603287581480964</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.5040798559587287</v>
+        <v>0.5262176839312582</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.4223100188112756</v>
+        <v>0.3432732210396773</v>
       </c>
     </row>
     <row r="18">
@@ -2339,21 +2339,21 @@
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Fácil</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.2781696602568258</v>
+        <v>0.09662790463757898</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.5058616126320689</v>
+        <v>0.5721618020221613</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3920156364444473</v>
+        <v>0.3343948533298701</v>
       </c>
     </row>
     <row r="19">
@@ -2366,7 +2366,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2374,13 +2374,13 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.1856148174867425</v>
+        <v>0.06226391921993668</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.5980001585399306</v>
+        <v>0.5689798253105696</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.3918074880133365</v>
+        <v>0.3156218722652531</v>
       </c>
     </row>
     <row r="20">
@@ -2393,7 +2393,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2401,13 +2401,13 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.2041277809699723</v>
+        <v>0.07391059869333683</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.535697686918587</v>
+        <v>0.5377050627497266</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.3699127339442796</v>
+        <v>0.3058078307215317</v>
       </c>
     </row>
     <row r="21">
@@ -2420,7 +2420,7 @@
         <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2428,13 +2428,13 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.3144355837463169</v>
+        <v>0.07578908151193076</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0.4204738342885873</v>
+        <v>0.5182309148646962</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.3674547090174521</v>
+        <v>0.2970099981883135</v>
       </c>
     </row>
     <row r="22">
@@ -2447,7 +2447,7 @@
         <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>68</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2455,13 +2455,13 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.1911099879500817</v>
+        <v>0.130494024462659</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0.5387368264886676</v>
+        <v>0.4520645623179925</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0.3649234072193747</v>
+        <v>0.2912792933903258</v>
       </c>
     </row>
     <row r="23">
@@ -2474,7 +2474,7 @@
         <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2482,13 +2482,13 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.2344513728229287</v>
+        <v>0.08976085058295136</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.4919808882021666</v>
+        <v>0.4919875173903151</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.3632161305125476</v>
+        <v>0.2908741839866332</v>
       </c>
     </row>
     <row r="24">
@@ -2501,7 +2501,7 @@
         <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2509,13 +2509,13 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.1833417569567551</v>
+        <v>0.03771985201661943</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.524841252334851</v>
+        <v>0.5432211448211409</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.3540915046458031</v>
+        <v>0.2904704984188802</v>
       </c>
     </row>
     <row r="25">
@@ -2528,7 +2528,7 @@
         <v>10</v>
       </c>
       <c r="C25" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2536,13 +2536,13 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.1552423791450023</v>
+        <v>0.1497035382653547</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0.5519061004696417</v>
+        <v>0.4241053607629135</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.353574239807322</v>
+        <v>0.2869044495141341</v>
       </c>
     </row>
   </sheetData>
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46256.98052083333</v>
+        <v>46237.90368055556</v>
       </c>
     </row>
     <row r="7">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/home/isaquenascimento/ast-driven-data-augmentation-algorithm/data/censo_escolar_dataset/augmentation_method_results/censo_escolar_algorithm_only_augmented.json</t>
+          <t>/home/ioolliver/Workspace/ast-driven-data-augmentation-algorithm/data/censo_escolar_dataset/augmentation_method_results/censo_escolar_algorithm_only_augmented.json</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Qwen/Qwen3-Embedding-4B</t>
+          <t>jinaai/jina-embeddings-v3</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>symmetric text similarity</t>
+          <t>text-matching</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Apache-2.0</t>
+          <t>CC BY-NC 4.0</t>
         </is>
       </c>
     </row>

</xml_diff>